<commit_message>
Bug Fixes in Windows
</commit_message>
<xml_diff>
--- a/question/gamemode_logic.xlsx
+++ b/question/gamemode_logic.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDHANT\Desktop\Zendalona\forkedFolder\Maths-Tutor-QT-V2\question\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F155D148-DA25-4FD4-B5F7-95F804454666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FA29BC-ADFC-4E39-A449-F430A23163F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>

</xml_diff>

<commit_message>
Bug FIxes on linux : 1.Restored a function for thread lock. \n2.gamemode_logic cleared.
</commit_message>
<xml_diff>
--- a/question/gamemode_logic.xlsx
+++ b/question/gamemode_logic.xlsx
@@ -17,6 +17,29 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t xml:space="preserve">label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">backward</t>
+  </si>
+  <si>
+    <t xml:space="preserve">warmup_order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">minimum_correct</t>
+  </si>
+  <si>
+    <t xml:space="preserve">maximum_wrong</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -287,9 +310,30 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="0" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Excel file conflit resolve
</commit_message>
<xml_diff>
--- a/question/gamemode_logic.xlsx
+++ b/question/gamemode_logic.xlsx
@@ -1,74 +1,56 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDHANT\Desktop\Zendalona\forkedFolder\Maths-Tutor-QT-V2\question\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEEBA8B-58F1-4119-A495-04C98C4673AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
-  <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
-    <t xml:space="preserve">label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">forward</t>
-  </si>
-  <si>
-    <t xml:space="preserve">backward</t>
-  </si>
-  <si>
-    <t xml:space="preserve">warmup_order</t>
-  </si>
-  <si>
-    <t xml:space="preserve">minimum_correct</t>
-  </si>
-  <si>
-    <t xml:space="preserve">maximum_wrong</t>
+    <t>label</t>
+  </si>
+  <si>
+    <t>forward</t>
+  </si>
+  <si>
+    <t>backward</t>
+  </si>
+  <si>
+    <t>warmup_order</t>
+  </si>
+  <si>
+    <t>minimum_correct</t>
+  </si>
+  <si>
+    <t>maximum_wrong</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -80,7 +62,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
@@ -88,84 +70,64 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:srgbClr val="000000"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -173,173 +135,272 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme>
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="50000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="35000">
               <a:schemeClr val="phClr">
                 <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:shade val="51000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
                 <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
         <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="40000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="40000">
               <a:schemeClr val="phClr">
                 <a:tint val="45000"/>
                 <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill>
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="80000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="30000"/>
+                <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed saved_state issue and added rules localization for english
</commit_message>
<xml_diff>
--- a/question/gamemode_logic.xlsx
+++ b/question/gamemode_logic.xlsx
@@ -1,61 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SIDDHANT\Desktop\Zendalona\forkedFolder\Maths-Tutor-QT-V2\question\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBEEBA8B-58F1-4119-A495-04C98C4673AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>label</t>
-  </si>
-  <si>
-    <t>forward</t>
-  </si>
-  <si>
-    <t>backward</t>
-  </si>
-  <si>
-    <t>warmup_order</t>
-  </si>
-  <si>
-    <t>minimum_correct</t>
-  </si>
-  <si>
-    <t>maximum_wrong</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -74,21 +47,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -376,28 +408,44 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>label</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>forward</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>backward</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>warmup_order</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>minimum_correct</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>maximum_wrong</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refactored gamemode scoring, fixed progression in gamemode, fixed accessibility, added user guide, added ctrl+s to announce all shortcuts, removed ghost code.
</commit_message>
<xml_diff>
--- a/question/gamemode_logic.xlsx
+++ b/question/gamemode_logic.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,6 +448,448 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1D_addition</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1D_subtraction</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1D_subtraction</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1D_multiplication</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1D_addition</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1D_multiplication</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1D_division</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1D_subtraction</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1D_division</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2D_addition</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1D_multiplication</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2D_addition</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2D_subtraction</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1D_division</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2D_subtraction</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2D_multiplication</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2D_addition</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2D_multiplication</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2D_division</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2D_subtraction</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2D_division</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3D_addition</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2D_multiplication</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>3D_addition</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>3D_subtraction</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2D_division</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>9</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>3D_subtraction</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>3D_multiplication</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3D_addition</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>10</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>3D_multiplication</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3D_division</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>3D_subtraction</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>11</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3D_division</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>4D_addition</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3D_multiplication</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4D_addition</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>4D_subtraction</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>3D_division</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E14" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>4D_subtraction</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>4D_multiplication</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>4D_addition</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>14</v>
+      </c>
+      <c r="E15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>4D_multiplication</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>4D_division</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>4D_subtraction</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>4D_division</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>mixed_operation</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>4D_multiplication</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>16</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>mixed_operation</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>NaN</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>4D_division</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>